<commit_message>
docs: update Sprint_Backlog to latest version (4 decisions 2026-09-22)
</commit_message>
<xml_diff>
--- a/docs/sprint/Sprint_Backlog.xlsx
+++ b/docs/sprint/Sprint_Backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FPT_Ky5\SWP\bmad swp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02354215-4856-44FC-92DF-60F8D0E36657}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{679236C9-C663-4EF9-B9D5-2EE84AEB62CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,15 +46,15 @@
     <t>From-To</t>
   </si>
   <si>
+    <t>Business Rules</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
     <t>Mô tả</t>
   </si>
   <si>
-    <t>Business Rules</t>
-  </si>
-  <si>
-    <t>Note</t>
-  </si>
-  <si>
     <t>Project Setup + API Contract</t>
   </si>
   <si>
@@ -73,12 +73,15 @@
     <t>22/09/2026 - 05/10/2026</t>
   </si>
   <si>
+    <t>• openapi.yaml là nguồn tra cứu duy nhất của API — muốn đổi API phải sửa contract trước khi code.</t>
+  </si>
+  <si>
+    <t>AD-2/3/8 · Spring Boot 4.1.1 (Java 21) + Vite React 19.3</t>
+  </si>
+  <si>
     <t>Dựng khung dự án (monorepo BE + FE) và chốt hợp đồng API: mọi API lấy từ openapi.yaml, muốn đổi phải sửa contract trước. Thống nhất chuẩn lỗi + phân trang.</t>
   </si>
   <si>
-    <t>AD-2/3/8 · Spring Boot 4.1.1 (Java 21) + Vite React 19.3</t>
-  </si>
-  <si>
     <t>DB Schema — Flyway V1 (model V3)</t>
   </si>
   <si>
@@ -91,19 +94,22 @@
     <t>—</t>
   </si>
   <si>
+    <t>• Tiền tệ lưu DECIMAL(15,0) — cấm float/double.
+• Mọi mốc thời gian lưu UTC hcm/asia.
+• ActivityLog chỉ được INSERT — không UPDATE, không DELETE.
+• Thay đổi schema chỉ qua migration Flyway — cấm DDL tay và hbm2ddl auto.</t>
+  </si>
+  <si>
+    <t>AD-6/7 · Flyway V1 · Thuần BE</t>
+  </si>
+  <si>
     <t>Tạo toàn bộ CSDL (22 bảng) theo model V3 bằng Flyway. Tiền lưu DECIMAL cấm float; nhật ký chỉ ghi thêm, không sửa/xóa.</t>
   </si>
   <si>
-    <t>AD-6/7 · Flyway V1 · Thuần BE</t>
-  </si>
-  <si>
     <t>Seed demo data</t>
   </si>
   <si>
     <t>Huy</t>
-  </si>
-  <si>
-    <t>Sinh dữ liệu demo: 5 quyền, user mẫu, kho Tân Bình + unit, bảng giá v3, dữ liệu lịch sử đủ chạy dashboard và demo 6 hành trình.</t>
   </si>
   <si>
     <t>• Seed phải đủ 5 role (kèm System Administrator) và user demo cho từng role.
@@ -113,10 +119,10 @@
     <t>Mã demo chuẩn: BK-1042, RT-0871, SR-0032, CT-1042, CT-1042-A1 · Thuần BE</t>
   </si>
   <si>
+    <t>Sinh dữ liệu demo: 5 quyền, user mẫu, kho Tân Bình + unit, bảng giá v3, dữ liệu lịch sử đủ chạy dashboard và demo 6 hành trình.</t>
+  </si>
+  <si>
     <t>Login + Adaptive Shell 5 role</t>
-  </si>
-  <si>
-    <t>Đăng nhập JWT: mỗi vai trò vào trang chủ riêng, sai thông tin báo lỗi chung, vào vùng khác vai trò bị 403. Phân quyền chặn ở server; ghi log mọi lần đăng nhập.</t>
   </si>
   <si>
     <t>• Phiên đăng nhập hiệu lực 24h (JWT) — không cấp refresh token.
@@ -130,6 +136,9 @@
     <t>FR-1, FR-38 · AD-5</t>
   </si>
   <si>
+    <t>Đăng nhập JWT: mỗi vai trò vào trang chủ riêng, sai thông tin báo lỗi chung, vào vùng khác vai trò bị 403. Phân quyền chặn ở server; ghi log mọi lần đăng nhập.</t>
+  </si>
+  <si>
     <t>Register + Forgot password</t>
   </si>
   <si>
@@ -137,150 +146,134 @@
   </si>
   <si>
     <t>Tuấn Anh</t>
-  </si>
-  <si>
-    <t>Đăng ký công khai chỉ tạo Customer, email trùng báo ngay. Quên mật khẩu trả lời chung chung, chưa gửi email thật.</t>
   </si>
   <si>
     <t>• Form đăng ký công khai chỉ tạo CUSTOMER — không có trường chọn role.
 • Email đã tồn tại → chặn, báo inline ngay tại form.
-• Đăng ký thành công → tự đăng nhập vào Browse Units.
-• Quên mật khẩu luôn trả phản hồi giống nhau dù email có tồn tại hay không.
-• Không gửi email thật trong v1 (P2).</t>
+• Quên mật khẩu luôn trả phản hồi giống nhau dù email có tồn tại hay không.</t>
   </si>
   <si>
     <t>FR-2, FR-3 (P2)</t>
   </si>
   <si>
+    <t>Đăng ký công khai chỉ tạo Customer, email trùng báo ngay. Quên mật khẩu trả lời chung chung, chưa gửi email thật.</t>
+  </si>
+  <si>
     <t>Browse Units + availability chính xác</t>
   </si>
   <si>
+    <t>• Unit Rented/Maintenance/Retired không xuất hiện trong kết quả.
+• tgian thuê được là không dính tgian thuê và ko dính tgian đệm, tính tại thời điểm query trên server
+• Sắp xếp mặc định: giá thấp → cao.</t>
+  </si>
+  <si>
+    <t>FR-4 · AD-4</t>
+  </si>
+  <si>
     <t>Danh sách unit dạng card: lọc loại/kích thước/ngày, sort theo giá. Còn trống tính trên server (đặt chỗ + buffer dọn); unit không cho thuê không hiện.</t>
   </si>
   <si>
-    <t>• Unit Rented/Maintenance/Retired không xuất hiện trong kết quả.
-• Availability = Reservation + Turnover Buffer, tính tại thời điểm query trên server — FE hiển thị nguyên văn, không tự tính lại.
-• Unit đang trong buffer dọn hiển thị ngày sẵn sàng và vẫn đặt được với ngày đó.
-• Chỉ làm mới danh sách khi bấm Search — không query theo từng phím gõ.
-• Sắp xếp mặc định: giá thấp → cao.</t>
-  </si>
-  <si>
-    <t>FR-4 · AD-4</t>
-  </si>
-  <si>
     <t>Unit Detail + bảng giá minh bạch</t>
   </si>
   <si>
+    <t>• Bảng giá phải đủ: rent × duration + từng dòng phụ thu theo Rental Policy đang hiệu lực.
+• tiền cọc hiển thị kèm nhãn refundable (hoàn lại).
+• Tiền hiển thị VND đầy đủ (1.150.000 ₫).</t>
+  </si>
+  <si>
+    <t>FR-6 · NFR-1</t>
+  </si>
+  <si>
     <t>Trang chi tiết unit + bảng giá minh bạch: tiền thuê, từng phụ thu, cọc ghi rõ hoàn lại. Số tiền khớp mọi màn sau; format tiền VND chuẩn.</t>
   </si>
   <si>
-    <t>• Bảng giá phải đủ: rent × duration + từng dòng phụ thu theo Rental Policy đang hiệu lực.
-• Deposit hiển thị kèm nhãn refundable (hoàn lại).
-• Mọi dòng tiền phải khớp tuyệt đối với Booking Summary và Payment Modal.
-• Tiền hiển thị VND full precision (1.150.000 ₫).</t>
-  </si>
-  <si>
-    <t>FR-6 · NFR-1</t>
-  </si>
-  <si>
     <t>Payment Modal + mock gateway</t>
-  </si>
-  <si>
-    <t>Một modal thanh toán dùng chung: Card / MoMo / VNPay QR. Đang xử lý không đóng được; lỗi đồng nghĩa chưa trừ tiền, được thử lại hoặc đổi cách; thành công có receipt vĩnh viễn.</t>
   </si>
   <si>
     <t>• Một modal dùng chung cho 4 điểm thanh toán: Deposit, 100% rent, Extension fee, Extra fee.
 • Hỗ trợ 3 phương thức: Card / MoMo (OTP) / VNPay QR (hết hạn sau ~5 phút).
 • Đang xử lý không được đóng modal hay điều hướng rời trang.
 • Thất bại = chưa trừ tiền, KHÔNG thay đổi trạng thái nào — khách được Retry hoặc đổi phương thức.
-• Sau 2 lần thất bại phải gợi ý đổi phương thức.
-• Mỗi payment thành công sinh đúng 1 receipt, xem được vĩnh viễn.
+• Mỗi payment thành công sinh đúng 1 hoá đơn, xem được vĩnh viễn.
 • Kết quả thanh toán chỉ do server (gateway) quyết định — FE không tự quyết.</t>
   </si>
   <si>
     <t>FR-8/9 · AD-9 (gateway interface + mock)</t>
   </si>
   <si>
+    <t>Một modal thanh toán dùng chung: Card / MoMo / VNPay QR. Đang xử lý không đóng được; lỗi đồng nghĩa chưa trừ tiền, được thử lại hoặc đổi cách; thành công có receipt vĩnh viễn.</t>
+  </si>
+  <si>
     <t>Booking Summary + Reserve re-check</t>
   </si>
   <si>
+    <t>• Booking Summary phải liệt kê 100% dòng tiền khách sẽ bị truy đòi — không dòng nào xuất hiện ở Payment mà vắng ở đây.
+• Bấm Reserve phải re-check availability — unit bị chiếm giữa chừng thì không được đặt, quay về trang tìm kiếm + gợi ý unit tương tự.</t>
+  </si>
+  <si>
+    <t>FR-5/7</t>
+  </si>
+  <si>
     <t>Trước khi trả cọc khách duyệt lại toàn bộ dòng tiền. Bấm Reserve hệ thống kiểm lại unit còn trống — bị giành thì quay về lưới kèm gợi ý; cọc xong unit được giữ.</t>
   </si>
   <si>
-    <t>• Booking Summary phải liệt kê 100% dòng tiền khách sẽ bị truy đòi — không dòng nào xuất hiện ở Payment mà vắng ở đây.
-• Hợp đồng draft chỉ sinh từ đúng các điều kiện đã duyệt tại đây.
-• Bấm Reserve phải re-check availability — unit bị chiếm giữa chừng thì không được đặt, quay về lưới + gợi ý unit tương tự.
-• Không bao giờ booking trên ngày không còn hiệu lực.
-• Reserve thành công → Reservation = PENDING_PAYMENT.
-• Deposit thành công → Reservation = RESERVED, unit bị giữ từ đây.</t>
-  </si>
-  <si>
-    <t>FR-5/7</t>
-  </si>
-  <si>
     <t>Reservation lifecycle + EXPIRED no-show</t>
-  </si>
-  <si>
-    <t>Quá hạn nhận kho mà không check-in → Reservation hết hạn: mất cọc, unit mở lại, đóng contract draft, báo khách. Hết hạn tính trên server.</t>
   </si>
   <si>
     <t>• Quá ngày nhận kho mà chưa check-in → Reservation = EXPIRED.
 • EXPIRED → khách mất cọc, receipt ghi "Deposit forfeited — no-show".
-• EXPIRED → Unit = Available; Contract Draft/Printed = Closed.
 • EXPIRED phải ghi ActivityLog + notification cho khách.
-• EXPIRED do server suy diễn on-read — API luôn trả state cuối, FE không tự suy từ ngày.
-• v1 không có cancel đặt chỗ.</t>
+• EXPIRED do server suy diễn on-read — API luôn trả state cuối, FE không tự suy từ ngày.</t>
   </si>
   <si>
     <t>FR-36 · AD-4 · Thuần BE</t>
   </si>
   <si>
+    <t>Quá hạn nhận kho mà không check-in → Reservation hết hạn: mất cọc, unit mở lại, đóng contract draft, báo khách. Hết hạn tính trên server.</t>
+  </si>
+  <si>
     <t>Contract auto-draft</t>
   </si>
   <si>
+    <t>• Contract Draft sinh tự động ngay khi Deposit thành công — không có đường sinh tay.
+• Contract luôn read-only — không UI nào cho phép sửa.
+• bản cũ chuyển thành `Superseded` , vẫn đọc được trong chuỗi.</t>
+  </si>
+  <si>
+    <t>FR-10/13 · Thuần BE</t>
+  </si>
+  <si>
     <t>Cọc thành công → tự động sinh hợp đồng draft, khóa phiên bản giá. Hợp đồng chỉ đọc; sai thì soạn lại, bản cũ vẫn xem được.</t>
   </si>
   <si>
-    <t>• Contract Draft sinh tự động ngay khi Deposit thành công — không có đường sinh tay.
-• Mã contract dạng CT-xxxx.
-• Mỗi contract khóa phiên bản Rental Policy tại thời điểm sinh.
-• Contract luôn read-only — không UI nào cho phép sửa.
-• Sửa draft = re-draft: bản cũ chuyển Superseded, vẫn đọc được trong chuỗi.</t>
-  </si>
-  <si>
-    <t>FR-10/13 · Thuần BE</t>
-  </si>
-  <si>
     <t>My Rentals + Check-in Pass</t>
-  </si>
-  <si>
-    <t>Khách xem danh sách đặt chỗ/thuê của mình + mã check-in BK- đưa staff kiểm tại quầy kèm hướng dẫn. Số liệu lấy từ nguồn, không tự tính.</t>
   </si>
   <si>
     <t>• My Rentals hiển thị đủ 3 nhóm: Reservations / Rentals / History, mỗi card có status badge + nút action kế tiếp.
 • Mọi số liệu/trạng thái lấy nguyên văn từ nguồn — FE không tự tính lại.
-• Mã đặt chỗ BK- hiển thị lớn (mono) để staff đối chiếu tại quầy.
-• Empty state chỉ có đúng 1 CTA trỏ về flow đổ dữ liệu.</t>
+• Mã đặt chỗ BK- hiển thị lớn (mono) để staff đối chiếu tại quầy.</t>
   </si>
   <si>
     <t>FR-35 · NFR-8</t>
   </si>
   <si>
+    <t>Khách xem danh sách đặt chỗ/thuê của mình + mã check-in BK- đưa staff kiểm tại quầy kèm hướng dẫn. Số liệu lấy từ nguồn, không tự tính.</t>
+  </si>
+  <si>
     <t>Rental Detail + contract chain</t>
   </si>
   <si>
+    <t>• Mỗi rental hiển thị: unit, dates, payment history, receipts, deposit status (held/settled).
+• Chuỗi hợp đồng: gốc + mọi phụ lục; bản Signed, Superseded xem được mãi.
+• Addendum chưa ký phải treo thông báo nêu deadline ký tại quầy.</t>
+  </si>
+  <si>
+    <t>FR-9/13/35</t>
+  </si>
+  <si>
     <t>Trang chi tiết một lần thuê: unit, ngày, lịch sử thanh toán, cọc, chuỗi hợp đồng + phụ lục. Mọi thao tác (check-in, gia hạn, trả kho, hỗ trợ) bắt đầu từ đây.</t>
   </si>
   <si>
-    <t>• Mỗi rental hiển thị: unit, dates, payment history, receipts vĩnh viễn, deposit status (held/settled).
-• Chuỗi contract: gốc + mọi addendum; bản Signed xem mãi; Superseded vẫn đọc được.
-• Addendum chưa ký phải có amber banner nêu deadline ký tại quầy.
-• Mọi action (Check-in, Extend, Checkout Request, New Support) chỉ bắt đầu từ đây — không flow nào bắt đầu từ system menu.</t>
-  </si>
-  <si>
-    <t>FR-9/13/35</t>
-  </si>
-  <si>
     <t>Task Board — kanban 5 loại card</t>
   </si>
   <si>
@@ -288,30 +281,26 @@
   </si>
   <si>
     <t>06/10/2026 - 19/10/2026</t>
-  </si>
-  <si>
-    <t>Kanban cho staff: To do / In progress / Done với 5 loại thẻ (check-in, checkout, dọn, hỗ trợ, ký hợp đồng); di chuyển bằng kéo thả hoặc phím.</t>
   </si>
   <si>
     <t>• Board đúng 3 cột: To do / In progress / Done.
 • Thẻ đúng 5 loại: Check-in / Checkout / Cleaning / Support / Contract-signature.
-• Thẻ sinh tự động theo ca trực (route theo Unit + shift).
-• Di chuyển thẻ bằng kéo thả HOẶC bàn phím — kéo thả không phải con đường duy nhất.
-• Thẻ Done hiển thị muted; số lượng từng cột hiển thị ở header.</t>
+• Mọi thẻ do hệ thống sinh từ sự kiện nghiệp vụ, route theo Unit + shift (kể cả task bảo trì/dọn phát sinh từ Severity Decision của Manager) — không có đường giao tay.
+• Mặc định: hiện thẻ trong ngày/ca hiện tại.</t>
   </si>
   <si>
     <t>FR-21 · NFR-2</t>
   </si>
   <si>
+    <t>Kanban cho staff: To do / In progress / Done với 5 loại thẻ (check-in, checkout, dọn, hỗ trợ, ký hợp đồng); di chuyển bằng kéo thả hoặc phím.</t>
+  </si>
+  <si>
     <t>Check-in Task — ritual hợp đồng</t>
-  </si>
-  <si>
-    <t>Check-in tại quầy: xác nhận reservation đã cọc → thu 100% tiền thuê → in hợp đồng, chụp ảnh bản ký → mới được trao access code.</t>
   </si>
   <si>
     <t>• Chỉ được check-in khi Reservation tồn tại VÀ Deposit đã thanh toán — vi phạm chặn kèm lý do cụ thể.
 • Deposit và 100% rent là 2 khoản thanh toán tách biệt.
-• Access code chỉ được trao sau khi có ảnh bản ký hợp đồng.
+• Access code chỉ được trao sau khi đã ký hợp đồng.
 • Đính kèm ảnh bản ký phải ghi CONTRACT_SIGNED vào ActivityLog.
 • Hoàn tất → Rental = CHECKED_IN, Unit = RENTED, task = Done.</t>
   </si>
@@ -319,119 +308,113 @@
     <t>FR-11/14/15</t>
   </si>
   <si>
+    <t>Check-in tại quầy: xác nhận reservation đã cọc → thu 100% tiền thuê → in hợp đồng, chụp ảnh bản ký → mới được trao access code.</t>
+  </si>
+  <si>
     <t>Snap-back chống Done ảo</t>
   </si>
   <si>
+    <t>• Thẻ chỉ được Done khi bước chốt đã xong (thanh toán / settlement / ảnh bản ký).</t>
+  </si>
+  <si>
+    <t>FR-22 · AD-4</t>
+  </si>
+  <si>
     <t>Kéo thẻ sang Done khi chưa xong bước chốt (thanh toán, ảnh ký...) → thẻ bật lại và báo thiếu bước nào. Không có Done ảo.</t>
   </si>
   <si>
-    <t>• Thẻ chỉ được Done khi bước chốt đã xong (thanh toán / settlement / ảnh bản ký).
-• Kéo sang Done khi thiếu bước chốt → thẻ bật lại + toast nêu đúng bước thiếu.
-• Rule enforce ở service — FE chỉ hiển thị kết quả.</t>
-  </si>
-  <si>
-    <t>FR-22 · AD-4</t>
-  </si>
-  <si>
     <t>Toast + Bell + Notification feed</t>
   </si>
   <si>
+    <t>• Toast tồn tại ~4s, hover pause, tối đa 1 action link.
+• Bell badge hiện số TB chưa đọc.
+• Feed theo vai trò: khách (booking/payment/support), staff (task assignment), manager (escalation + status writes).</t>
+  </si>
+  <si>
+    <t>FR-33/34</t>
+  </si>
+  <si>
     <t>Thông báo: toast ngắn ~4s + chuông có badge số chưa đọc; feed theo vai trò, bấm vào tới thẳng đối tượng. Không gửi email.</t>
   </si>
   <si>
-    <t>• Toast tồn tại ~4s, hover pause, tối đa 1 action link.
-• Bell badge đếm số chưa đọc; unread persist giữa các phiên.
-• Feed theo vai trò: khách (booking/payment/support), staff (task assignment), manager (escalation + status writes).
-• Sự kiện liên quan tiền phải phát cả toast lẫn bell.
-• Feed sắp unread trước, deep link tới đối tượng.
-• Không gửi email — không bao giờ.</t>
-  </si>
-  <si>
-    <t>FR-33/34</t>
-  </si>
-  <si>
     <t>Extension + conflict boundary</t>
-  </si>
-  <si>
-    <t>Gia hạn: khách chọn ngày trả mới, chặn nếu đụng đặt chỗ kế tiếp (báo rõ ngày giới hạn). Phí = tiền thuê kỳ thêm theo giá đang hiệu lực; trả xong cập nhật ngày + sinh phụ lục.</t>
   </si>
   <si>
     <t>• Ngày checkout mới không được đụng Reservation kế tiếp — submit bị chặn kèm biên rõ ("Latest new checkout: Oct 18").
 • Extension chỉ mở TRƯỚC EndDate hiện tại.
-• Quá EndDate: giữ CHECKED_IN, không có trạng thái OVERDUE — mỗi ngày trễ tính LATE_FEE lúc settlement.
-• Phí gia hạn = tiền thuê kỳ thêm theo Rental Policy đang hiệu lực (không dùng hiệu số cọc).
-• Deposit giữ nguyên booking gốc.
-• Thanh toán thành công → EndDate cập nhật NGAY + sinh Addendum.</t>
-  </si>
-  <si>
-    <t>FR-16/12 · Trễ không có trạng thái OVERDUE — tính LATE_FEE lúc tất toán</t>
+• Phí gia hạn = tiền thuê kỳ thêm theo Rental Policy đang hiệu lực + top-up cọc = max(0, Deposit% × tổng tiền thuê hợp đồng sau gia hạn − cọc đang giữ).
+• Thanh toán thành công → EndDate cập nhật NGAY, cọc đang giữ nâng lên mức mới, sinh Addendum (ghi số cọc mới).
+• Settlement dùng số cọc hiện giữ — công thức refund không đổi.</t>
+  </si>
+  <si>
+    <t>FR-16/12 · Trễ không có OVERDUE — tính LATE_FEE lúc tất toán · Top-up cọc chốt 2026-09-22 (demo: 690.000 + 69.000 = 759.000 ₫, cọc → 172.500 ₫)</t>
+  </si>
+  <si>
+    <t>Gia hạn: khách chọn ngày trả mới, chặn nếu đụng đặt chỗ kế tiếp (báo rõ ngày giới hạn). Phí = tiền thuê kỳ thêm + top-up cọc về mức mới theo giá đang hiệu lực; trả xong cập nhật ngày + cọc + sinh phụ lục.</t>
   </si>
   <si>
     <t>Addendum giấy + Contract-signature card</t>
   </si>
   <si>
-    <t>Phụ lục gia hạn CT-…-A1: hẹn ký tại quầy 7 ngày, nhắc cả 2 bên; ký xong ảnh vào hồ sơ. Quá hạn chỉ nhắc mạnh hơn, không thu hồi ngày.</t>
-  </si>
-  <si>
-    <t>• Addendum (CT-…-A1) sinh sau khi trả phí gia hạn.
+    <t>• Addendum (CT-…-A1) sinh tự động sau khi trả phí gia hạn — không có đường sinh tay nên không tồn tại ca "soạn nhầm" (khác hợp đồng gốc có re-draft).
+• Addendum không hold Unit — ngày mới hiệu lực ngay từ lúc trả phí, phụ lục chỉ là hồ sơ giấy.
 • Deadline ký tại quầy: 7 ngày.
 • Trạng thái AWAITING_SIGNATURE cho đến khi có ảnh bản ký → SIGNED.
 • Nút hoàn tất ký vô hiệu đến khi capture tile có ảnh.
-• Quá deadline → reminder tăng cường, KHÔNG thu hồi ngày.
-• Addendum không hold Unit.
-• Addendum Voided (soạn nhầm/trả sớm) → soạn lại thành bản ghi mới của cùng Extension.</t>
-  </si>
-  <si>
-    <t>FR-12</t>
+• Voided chỉ còn 1 đường: khách trả kho sớm trước khi ký → staff đóng hồ sơ, không soạn lại.</t>
+  </si>
+  <si>
+    <t>FR-12 · Chốt 2026-09-22: bỏ trigger "soạn nhầm", giữ Voided cho trả kho sớm</t>
+  </si>
+  <si>
+    <t>Phụ lục gia hạn CT-…-A1: hẹn ký tại quầy 7 ngày, nhắc cả 2 bên; ký xong ảnh vào hồ sơ. Quá hạn chỉ nhắc mạnh hơn, không thu hồi ngày.</t>
   </si>
   <si>
     <t>Checkout Request</t>
-  </si>
-  <si>
-    <t>Khách xin trả kho ngay trên trang rental → sinh thẻ Checkout cho staff; request mới thay request cũ.</t>
   </si>
   <si>
     <t>• Checkout request gửi từ Rental Detail, kèm giải thích logic tất toán (hoàn / trừ / thu thêm).
 • Gửi thành công → Rental = CHECKOUT_REQUESTED + sinh Checkout Task.
 • Request mới thay request cũ — request cũ tự hủy.
-• Request chỉ DONE khi settlement hoàn tất.
-• Ngày xin trả bị chặn trên biên Reservation kế tiếp (như Extension).</t>
+• Request chỉ DONE khi settlement hoàn tất.</t>
   </si>
   <si>
     <t>FR-17</t>
   </si>
   <si>
+    <t>Khách xin trả kho ngay trên trang rental → sinh thẻ Checkout cho staff; request mới thay request cũ.</t>
+  </si>
+  <si>
     <t>Checkout Task — climax tất toán</t>
   </si>
   <si>
+    <t>• Nhận Unit + key theo checklist; Inspection từng hạng mục (access card, padlock, cleanliness, structure) với kết quả OK/MINOR/MAJOR. 
+• Charge damage bắt buộc có số tiền + reason.
+• Settlement = Deposit − charges = refund; tiền hư hao vượt tiền cọc → khách trả phần chênh.
+• Không đóng rental khi còn charge thiếu reason hoặc phần chênh chưa trả.
+• Settlement receipt hiển thị 2 bên.
+• Đóng rental → Unit = Preparing + sinh Cleaning Task.</t>
+  </si>
+  <si>
+    <t>FR-18</t>
+  </si>
+  <si>
     <t>Staff nhận unit: checklist, kiểm tra hạng mục, kê khai phụ phí kèm lý do bắt buộc → tất toán (hoàn cọc hoặc thu thêm) → đóng rental, sinh thẻ dọn.</t>
   </si>
   <si>
-    <t>• Nhận Unit + key theo checklist; Inspection từng hạng mục (access card, padlock, cleanliness, structure) với kết quả OK/MINOR/MAJOR.
-• Charge damage bắt buộc có số tiền + reason.
-• Settlement = Deposit − charges = refund; charges vượt Deposit → khách trả phần chênh (touchpoint Extra fee).
-• Không đóng rental khi còn charge thiếu reason hoặc phần chênh chưa trả.
-• Settlement receipt hiển thị 2 bên vĩnh viễn.
-• Đóng rental → Unit = Preparing + sinh Cleaning Task.</t>
-  </si>
-  <si>
-    <t>FR-18</t>
-  </si>
-  <si>
     <t>Cleaning + Turnover buffer</t>
   </si>
   <si>
+    <t>• Cleaning hoàn tất ngay trên thẻ — không màn hình riêng.
+• Unit chỉ rời Preparing khi thời gian đệm đã đủ.</t>
+  </si>
+  <si>
+    <t>FR-19</t>
+  </si>
+  <si>
     <t>Hoàn tất dọn ngay trên thẻ; unit chỉ mở cho thuê khi đủ ngày buffer theo policy.</t>
   </si>
   <si>
-    <t>• Cleaning hoàn tất ngay trên thẻ — không màn hình riêng.
-• Unit chỉ rời Preparing khi Turnover Buffer đã đủ ngày theo policy.
-• Hết buffer → Unit = Available, hoặc Reserved nếu có Reservation kế.</t>
-  </si>
-  <si>
-    <t>FR-19</t>
-  </si>
-  <si>
     <t>Support Ticket — tạo, route, resolve/escalate</t>
   </si>
   <si>
@@ -441,42 +424,37 @@
     <t>20/10/2026 - 02/11/2026</t>
   </si>
   <si>
-    <t>Khách gửi ticket gắn với unit; hệ thống chuyển cho staff trực ca. Staff xử lý kèm ghi chú hoặc chuyển lên quản lý (escalate phải có ghi chú).</t>
-  </si>
-  <si>
-    <t>• Ticket bắt buộc: Unit hợp lệ + incident type (LOST_ACCESS/DEVICE_ISSUE/SECURITY/CLEANLINESS/OTHER) + mô tả.
+    <t xml:space="preserve">• Ticket bắt buộc: Unit hợp lệ + incident type (LOST_ACCESS/DEVICE_ISSUE/SECURITY/CLEANLINESS/OTHER) + mô tả.
 • Không có Unit hợp lệ → không gửi được.
 • Ticket route tự động tới staff trực ca theo Unit + shift.
 • Resolve phải kèm note — khách nhận kết quả plain words.
-• Escalate bắt buộc note (không note → nút vô hiệu) → vào Escalation Inbox của Facility Manager.</t>
+• Escalate bắt buộc note </t>
   </si>
   <si>
     <t>FR-23/24</t>
   </si>
   <si>
+    <t>Khách gửi ticket gắn với unit; hệ thống chuyển cho staff trực ca. Staff xử lý kèm ghi chú hoặc chuyển lên quản lý (escalate phải có ghi chú).</t>
+  </si>
+  <si>
     <t>Severity Decision + Relocation</t>
   </si>
   <si>
+    <t>• đổi trạng thái unit sang Maintenance.
+• Relocation = đổi unit trên Rental hiện tại: giữ mã RT-/Contract/Deposit — không sinh Rental mới.
+• Relocation: access code mới + ActivityLog RELOCATION + tasks bảo trì/dọn dẹp lên kanban + notification khách hàng.</t>
+  </si>
+  <si>
+    <t>FR-25</t>
+  </si>
+  <si>
     <t>Quản lý đánh giá ticket: nghiêm trọng → unit chuyển bảo trì + chuyển khách sang unit khác ngay trên rental hiện tại (giữ hợp đồng, cọc); nhẹ → trả về staff.</t>
   </si>
   <si>
-    <t>• Đánh dấu severe → Unit = Maintenance.
-• Relocation = đổi unit trên Rental hiện tại: giữ mã RT-/Contract/Deposit — không sinh Rental mới.
-• Relocation: access code mới + ActivityLog RELOCATION + tasks bảo trì/dọn về kanban + notification khách từng bước.
-• Không severe → ticket về lại staff kèm hướng dẫn.
-• Sau Severity Decision ticket luôn quay IN_PROGRESS — chỉ Resolved khi staff hoàn tất + note.</t>
-  </si>
-  <si>
-    <t>FR-25</t>
-  </si>
-  <si>
     <t>Unit Management + edit drawer + guards</t>
   </si>
   <si>
-    <t>Quản lý unit: sửa thông tin, gộp, cho nghỉ, bảo trì — đều có xác nhận và chặn khi unit còn được giữ/thuê; mọi thao tác ghi log.</t>
-  </si>
-  <si>
-    <t>• Merge chỉ khi không có Rental/Reservation active ở cả 2 unit + confirm "cannot be undone".
+    <t>• Merge 2 unit → P2, KHÔNG build (chốt 2026-09-22 — cắt không phá flow; beat demo UJ-4 thay bằng Retire S-2, vẫn demo đủ guard + blocker + confirm).
 • Mọi chuyển trạng thái unit qua guard + confirm — không silent status write.
 • Fix status bắt buộc reason.
 • Bị chặn → blocker nêu tên + link.
@@ -484,26 +462,26 @@
 • Mọi thao tác ghi Activity Log.</t>
   </si>
   <si>
-    <t>FR-26/20</t>
+    <t>FR-26/20 · Merge → P2 2026-09-22</t>
+  </si>
+  <si>
+    <t>Quản lý unit: sửa thông tin, cho nghỉ, bảo trì, sửa trạng thái — đều có xác nhận và chặn khi unit còn được giữ/thuê; mọi thao tác ghi log. (Merge 2 unit: P2 — không build.)</t>
   </si>
   <si>
     <t>Staff &amp; Shifts + conflict detection</t>
   </si>
   <si>
+    <t>• Phân công theo Staff × Zone × Ca (MORNING/AFTERNOON/EVENING) × ngày.
+• Không lưu phân công trùng người-ca-ngày — chặn trước khi SAVE, báo lỗi cụ thể.</t>
+  </si>
+  <si>
+    <t>FR-27</t>
+  </si>
+  <si>
     <t>Phân công staff theo khu vực × ca × ngày trên lịch tuần; trùng người-ca-ngày bị chặn trước khi lưu, báo cụ thể.</t>
   </si>
   <si>
-    <t>• Phân công theo Staff × Zone × Ca (MORNING/AFTERNOON/EVENING) × ngày.
-• Không lưu phân công trùng người-ca-ngày — chặn trước khi SAVE, báo collision cụ thể.</t>
-  </si>
-  <si>
-    <t>FR-27</t>
-  </si>
-  <si>
     <t>Activity Log viewer</t>
-  </si>
-  <si>
-    <t>Xem nhật ký hệ thống (ai làm gì, khi nào, vì sao) chỉ đọc, lọc theo đối tượng; không xóa/sửa được.</t>
   </si>
   <si>
     <t>• Mỗi dòng log: timestamp, actor, entity, action, from → to, reason (nơi bắt buộc).
@@ -514,10 +492,10 @@
     <t>FR-28 · NFR-6</t>
   </si>
   <si>
+    <t>Xem nhật ký hệ thống (ai làm gì, khi nào, vì sao) chỉ đọc, lọc theo đối tượng; không xóa/sửa được.</t>
+  </si>
+  <si>
     <t>User Management — SYS-01</t>
-  </si>
-  <si>
-    <t>SysAdmin quản lý user: tạo tài khoản mọi vai trò, đổi vai trò, khóa/mở, reset mật khẩu. Không xóa user — chỉ đổi trạng thái; không tự khóa chính mình.</t>
   </si>
   <si>
     <t>• Tạo được tài khoản cho mọi role, kèm mật khẩu tạm.
@@ -525,20 +503,19 @@
 • Trạng thái user chỉ 0/1/2 (deactivate/active/lock) — KHÔNG xóa user.
 • Reset password = cấp mật khẩu tạm mới.
 • Email trùng → chặn inline.
-• Không được tự khóa chính mình.
-• Đăng nhập bằng tài khoản deactivate/lock → message chung, không tiết lộ lý do.</t>
+• Không được tự khóa chính mình.</t>
   </si>
   <si>
     <t>FR-37</t>
   </si>
   <si>
+    <t>SysAdmin quản lý user: tạo tài khoản mọi vai trò, đổi vai trò, khóa/mở, reset mật khẩu. Không xóa user — chỉ đổi trạng thái; không tự khóa chính mình.</t>
+  </si>
+  <si>
     <t>Login &amp; Activity History — SYS-02 + Permission matrix</t>
   </si>
   <si>
-    <t>Xem lịch sử đăng nhập (thành/bại) + bảng quyền vai trò × chức năng đúng như server đang chặn, chỉ đọc.</t>
-  </si>
-  <si>
-    <t>• Hiển thị LOGIN/LOGIN_FAILED với actor, thời điểm, kết quả; filter theo user/thời gian/kết quả.
+    <t>• Hiển thị LOGIN/LOGIN_FAILED với actor, thời điểm, kết quả; filter theo user/thời gian/kết quả. (cái hiển thị log của login được ko này có cần thiết ko, check lại đề)
 • Permission matrix Role × Permission hiển thị đúng như server enforce.
 • Matrix read-only — không chỉnh runtime; không tự tính lại nguồn.</t>
   </si>
@@ -546,27 +523,26 @@
     <t>FR-38/39</t>
   </si>
   <si>
+    <t>Xem lịch sử đăng nhập (thành/bại) + bảng quyền vai trò × chức năng đúng như server đang chặn, chỉ đọc.</t>
+  </si>
+  <si>
     <t>Policy Management — validate trước khi lưu</t>
   </si>
   <si>
-    <t>Sửa bảng giá quy định (giá cơ bản, phụ thu, % cọc, buffer ngày). Lưu luôn chạy validation — policy sai không bao giờ lưu được; lưu xong đóng dấu phiên bản + ngày hiệu lực.</t>
-  </si>
-  <si>
-    <t>• Chỉnh inline: base rent theo Unit Type, phụ thu + trần, Deposit %, Turnover Buffer ngày.
+    <t xml:space="preserve">• Chỉnh inline: base rent theo Unit Type, phụ thu + trần, Deposit %, Turnover Buffer ngày.
 • Save luôn chạy validation — giá trị vi phạm bị cắm cờ + banner nêu đúng luật ("15% exceeds the 10% cap in Rental Policy v3").
 • Policy không hợp lệ không bao giờ được persist.
 • Save thành công → đóng dấu version + effective date.
-• Đổi buffer/deposit chỉ ảnh hưởng tính toán từ phiên bản effective.
-• Block server hiển thị banner đầu form — không dùng toast.</t>
+</t>
   </si>
   <si>
     <t>FR-29/30 · NFR-8</t>
   </si>
   <si>
+    <t>Sửa bảng giá quy định (giá cơ bản, phụ thu, % cọc, buffer ngày). Lưu luôn chạy validation — policy sai không bao giờ lưu được; lưu xong đóng dấu phiên bản + ngày hiệu lực.</t>
+  </si>
+  <si>
     <t>Business Overview + Reports + KPI drill-down</t>
-  </si>
-  <si>
-    <t>Dashboard kinh doanh: KPI doanh thu / cọc đang giữ / phụ thu / công suất + báo cáo theo kỳ, export CSV; bấm KPI xuyên xuống bảng chi tiết.</t>
   </si>
   <si>
     <t>• KPI: revenue / deposits held / surcharges / utilization.
@@ -578,10 +554,10 @@
     <t>FR-31</t>
   </si>
   <si>
+    <t>Dashboard kinh doanh: KPI doanh thu / cọc đang giữ / phụ thu / công suất + báo cáo theo kỳ, export CSV; bấm KPI xuyên xuống bảng chi tiết.</t>
+  </si>
+  <si>
     <t>Facility Overview + drill-down</t>
-  </si>
-  <si>
-    <t>Dashboard vận hành: công suất, cơ cấu doanh thu, trạng thái unit; drill-down (VD occupancy 87% → danh sách unit đang thuê).</t>
   </si>
   <si>
     <t>• KPI occupancy / revenue mix / unit-status.
@@ -592,51 +568,47 @@
     <t>FR-32</t>
   </si>
   <si>
+    <t>Dashboard vận hành: công suất, cơ cấu doanh thu, trạng thái unit; drill-down (VD occupancy 87% → danh sách unit đang thuê).</t>
+  </si>
+  <si>
     <t>E2E Demo 6 UJ + deploy + hardening</t>
   </si>
   <si>
     <t>Cả nhóm</t>
-  </si>
-  <si>
-    <t>Chạy demo trọn 6 hành trình + test các ca bị ép (thiếu lý do charge, policy xấu, Done ảo...) + chốt môi trường deploy + rà NFR.</t>
   </si>
   <si>
     <t>• 6 UJ phải chạy trọn trên môi trường demo với seed chuẩn, không đứt gãy.
 • Test bắt buộc các ca ép: charge thiếu reason, policy xấu lưu, card Done thiếu bước, trao access code khi thiếu ảnh ký.
-• NFR phải rà: VND full precision, microcopy 3 phần, a11y floor (label, focus, keyboard, status không chỉ màu).
-• P2 đã cắt: Operations Monitor, notification day-grouping, Discount (FR-40), Waiver (FR-41) — cắt không phá flow.</t>
+• NFR phải rà: VND full precision (label, focus, keyboard, status không chỉ màu).
+• P2 đã cắt: Operations Monitor, notification day-grouping,  — cắt không phá flow.</t>
   </si>
   <si>
     <t>SM-1/2 · P2 đã cắt: Discount (FR-40), Waiver (FR-41), Operations Monitor</t>
   </si>
   <si>
-    <t>• openapi.yaml là nguồn tra cứu duy nhất của API — muốn đổi API phải sửa contract trước khi code.
-• Mọi lỗi trả về theo cú pháp chung: machine code + message + field errors.
-• Mọi danh sách trả về {items, page, pageSize, total}, mặc định 25 dòng/trang.</t>
-  </si>
-  <si>
-    <t>• Tiền tệ lưu DECIMAL(15,0) — cấm float/double.
-• Mọi mốc thời gian lưu UTC hcm/asia.
-• ActivityLog chỉ được INSERT — không UPDATE, không DELETE.
-• Thay đổi schema chỉ qua migration Flyway — cấm DDL tay và hbm2ddl auto.</t>
+    <t>Chạy demo trọn 6 hành trình + test các ca bị ép (thiếu lý do charge, policy xấu, Done ảo...) + chốt môi trường deploy + rà NFR.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -657,8 +629,13 @@
       <color rgb="FF548235"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFCC0000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -668,25 +645,42 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF305496"/>
+        <bgColor rgb="FF305496"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFDDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -713,41 +707,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -760,20 +760,20 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Sheets">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="4F81BD"/>
@@ -797,77 +797,19 @@
         <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="0000FF"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Sheets">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -879,160 +821,131 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="35000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="103000"/>
+                <a:lumMod val="102000"/>
+                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
+                <a:satMod val="110000"/>
+                <a:lumMod val="100000"/>
+                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="63000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr">
+            <a:tint val="95000"/>
+            <a:satMod val="170000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="93000"/>
+                <a:satMod val="150000"/>
+                <a:shade val="98000"/>
+                <a:lumMod val="102000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="40000">
+            <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
+                <a:tint val="98000"/>
+                <a:satMod val="130000"/>
+                <a:shade val="90000"/>
+                <a:lumMod val="103000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
+                <a:shade val="63000"/>
+                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1044,8 +957,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J34"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:J1000"/>
+  <sheetFormatPr defaultColWidth="14.3984375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
@@ -1056,9 +969,10 @@
     <col min="8" max="8" width="78" customWidth="1"/>
     <col min="9" max="9" width="34" customWidth="1"/>
     <col min="10" max="10" width="52" customWidth="1"/>
+    <col min="11" max="26" width="8.73046875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1081,16 +995,16 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="57" x14ac:dyDescent="0.45">
+    </row>
+    <row r="2" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1113,13 +1027,13 @@
         <v>15</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>156</v>
+        <v>16</v>
       </c>
       <c r="I2" s="5" t="s">
         <v>17</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="57" x14ac:dyDescent="0.45">
@@ -1127,16 +1041,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>14</v>
@@ -1145,13 +1059,13 @@
         <v>15</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>157</v>
+        <v>23</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
@@ -1159,16 +1073,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>14</v>
@@ -1177,13 +1091,13 @@
         <v>15</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
@@ -1191,10 +1105,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>12</v>
@@ -1209,30 +1123,30 @@
         <v>15</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="71.25" x14ac:dyDescent="0.45">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>14</v>
@@ -1241,30 +1155,30 @@
         <v>15</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>14</v>
@@ -1273,30 +1187,30 @@
         <v>15</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="57" x14ac:dyDescent="0.45">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>14</v>
@@ -1305,24 +1219,24 @@
         <v>15</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="114" x14ac:dyDescent="0.45">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>12</v>
@@ -1337,30 +1251,30 @@
         <v>15</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="114" x14ac:dyDescent="0.45">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>14</v>
@@ -1369,30 +1283,30 @@
         <v>15</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>14</v>
@@ -1401,30 +1315,30 @@
         <v>15</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="71.25" x14ac:dyDescent="0.45">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>14</v>
@@ -1433,27 +1347,27 @@
         <v>15</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="71.25" x14ac:dyDescent="0.45">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>13</v>
@@ -1464,28 +1378,28 @@
       <c r="G13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>65</v>
+      <c r="H13" s="8" t="s">
+        <v>66</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J13" s="5" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>13</v>
@@ -1497,13 +1411,13 @@
         <v>15</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="71.25" x14ac:dyDescent="0.45">
@@ -1511,31 +1425,31 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>72</v>
+        <v>37</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J15" s="5" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
@@ -1543,95 +1457,95 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>72</v>
+        <v>37</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F17" s="8" t="s">
-        <v>72</v>
+        <v>37</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="8" t="s">
-        <v>72</v>
+      <c r="F18" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J18" s="5" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="114" x14ac:dyDescent="0.45">
@@ -1639,10 +1553,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>12</v>
@@ -1650,20 +1564,20 @@
       <c r="E19" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F19" s="8" t="s">
-        <v>72</v>
+      <c r="F19" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
@@ -1671,10 +1585,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>12</v>
@@ -1682,212 +1596,212 @@
       <c r="E20" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F20" s="8" t="s">
-        <v>72</v>
+      <c r="F20" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="71.25" x14ac:dyDescent="0.45">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A21" s="2">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F21" s="8" t="s">
-        <v>72</v>
+      <c r="F21" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="114" x14ac:dyDescent="0.45">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A22" s="2">
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>72</v>
+        <v>37</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A23" s="2">
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>72</v>
+        <v>37</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>74</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I23" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A24" s="2">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F24" s="9" t="s">
-        <v>110</v>
+      <c r="F24" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A25" s="2">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>110</v>
+        <v>37</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="I25" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
       <c r="A26" s="2">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>110</v>
+        <v>37</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>121</v>
+        <v>113</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>122</v>
       </c>
       <c r="I26" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="J26" s="5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="28.5" x14ac:dyDescent="0.45">
@@ -1895,31 +1809,31 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>110</v>
+        <v>37</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I27" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J27" s="5" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
@@ -1927,39 +1841,39 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F28" s="9" t="s">
-        <v>110</v>
+      <c r="F28" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I28" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J28" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A29" s="2">
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>11</v>
@@ -1970,84 +1884,84 @@
       <c r="E29" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F29" s="9" t="s">
-        <v>110</v>
+      <c r="F29" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I29" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J29" s="5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="57" x14ac:dyDescent="0.45">
       <c r="A30" s="2">
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F30" s="9" t="s">
-        <v>110</v>
+      <c r="F30" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I30" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="J30" s="5" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="85.5" x14ac:dyDescent="0.45">
       <c r="A31" s="2">
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F31" s="9" t="s">
-        <v>110</v>
+      <c r="F31" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I31" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J31" s="5" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="57" x14ac:dyDescent="0.45">
@@ -2055,31 +1969,31 @@
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>110</v>
+        <v>37</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I32" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="42.75" x14ac:dyDescent="0.45">
@@ -2087,68 +2001,1034 @@
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>11</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F33" s="9" t="s">
-        <v>110</v>
+        <v>37</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I33" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J33" s="5" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="99.75" x14ac:dyDescent="0.45">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A34" s="2">
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F34" s="9" t="s">
-        <v>110</v>
+        <v>154</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>112</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I34" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J34" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="36" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="37" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="38" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="39" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="40" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="41" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="42" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="43" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="44" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="45" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="46" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="47" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="48" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="52" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="53" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="54" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="55" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="56" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="57" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="58" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="59" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="60" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="61" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="62" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="63" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="64" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="68" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="69" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="70" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="71" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="72" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="73" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="74" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="75" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="76" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="77" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="78" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="79" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="80" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="81" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="82" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="83" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="84" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="85" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="86" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="87" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="88" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="89" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="90" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="91" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="92" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="93" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="94" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="95" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="96" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="97" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="98" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="99" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="100" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="101" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="102" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="103" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="104" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="105" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="106" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="107" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="108" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="109" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="110" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="111" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="112" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="113" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="114" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="115" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="116" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="117" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="118" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="119" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="120" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="121" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="122" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="123" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="124" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="125" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="126" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="127" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="128" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="129" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="130" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="131" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="132" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="133" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="134" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="135" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="136" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="137" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="138" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="139" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="140" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="141" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="142" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="143" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="144" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="145" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="146" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="147" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="148" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="149" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="150" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="151" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="152" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="153" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="154" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="155" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="156" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="157" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="158" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="159" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="160" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="161" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="162" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="163" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="164" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="165" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="166" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="167" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="168" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="169" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="170" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="171" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="172" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="173" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="174" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="175" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="176" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="177" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="178" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="179" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="180" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="181" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="182" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="183" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="184" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="185" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="186" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="187" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="188" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="189" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="190" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="191" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="192" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="193" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="194" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="195" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="196" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="197" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="198" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="199" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="200" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="201" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="202" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="203" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="204" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="205" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="206" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="207" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="208" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="209" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="210" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="211" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="212" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="213" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="214" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="215" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="216" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="217" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="218" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="219" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="220" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="221" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="222" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="223" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="224" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="225" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="226" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="227" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="228" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="229" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="230" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="231" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="232" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="233" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="234" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="235" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="236" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="237" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="238" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="239" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="240" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="241" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="242" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="243" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="244" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="245" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="246" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="247" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="248" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="249" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="250" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="251" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="252" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="253" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="254" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="255" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="256" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="257" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="258" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="259" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="260" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="261" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="262" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="263" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="264" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="265" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="266" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="267" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="268" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="269" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="270" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="271" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="272" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="273" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="274" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="275" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="276" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="277" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="278" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="279" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="280" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="281" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="282" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="283" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="284" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="285" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="286" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="287" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="288" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="289" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="290" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="291" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="292" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="293" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="294" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="295" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="296" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="297" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="298" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="299" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="300" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="301" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="302" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="303" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="304" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="305" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="306" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="307" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="308" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="309" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="310" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="311" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="312" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="313" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="314" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="315" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="316" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="317" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="318" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="319" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="320" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="321" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="322" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="323" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="324" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="325" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="326" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="327" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="328" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="329" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="330" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="331" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="332" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="333" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="334" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="335" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="336" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="337" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="338" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="339" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="340" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="341" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="342" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="343" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="344" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="345" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="346" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="347" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="348" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="349" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="350" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="351" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="352" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="353" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="354" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="355" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="356" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="357" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="358" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="359" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="360" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="361" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="362" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="363" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="364" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="365" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="366" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="367" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="368" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="369" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="370" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="371" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="372" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="373" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="374" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="375" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="376" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="377" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="378" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="379" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="380" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="381" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="382" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="383" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="384" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="385" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="386" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="387" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="388" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="389" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="390" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="391" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="392" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="393" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="394" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="395" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="396" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="397" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="398" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="399" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="400" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="401" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="402" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="403" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="404" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="405" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="406" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="407" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="408" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="409" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="410" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="411" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="412" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="413" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="414" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="415" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="416" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="417" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="418" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="419" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="420" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="421" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="422" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="423" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="424" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="425" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="426" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="427" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="428" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="429" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="430" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="431" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="432" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="433" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="434" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="435" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="436" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="437" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="438" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="439" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="440" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="441" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="442" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="443" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="444" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="445" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="446" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="447" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="448" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="449" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="450" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="451" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="452" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="453" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="454" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="455" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="456" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="457" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="458" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="459" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="460" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="461" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="462" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="463" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="464" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="465" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="466" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="467" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="468" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="469" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="470" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="471" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="472" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="473" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="474" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="475" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="476" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="477" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="478" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="479" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="480" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="481" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="482" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="483" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="484" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="485" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="486" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="487" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="488" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="489" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="490" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="491" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="492" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="493" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="494" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="495" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="496" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="497" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="498" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="499" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="500" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="501" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="502" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="503" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="504" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="505" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="506" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="507" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="508" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="509" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="510" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="511" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="512" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="513" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="514" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="515" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="516" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="517" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="518" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="519" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="520" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="521" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="522" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="523" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="524" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="525" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="526" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="527" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="528" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="529" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="530" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="531" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="532" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="533" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="534" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="535" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="536" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="537" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="538" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="539" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="540" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="541" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="542" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="543" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="544" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="545" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="546" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="547" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="548" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="549" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="550" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="551" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="552" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="553" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="554" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="555" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="556" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="557" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="558" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="559" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="560" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="561" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="562" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="563" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="564" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="565" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="566" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="567" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="568" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="569" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="570" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="571" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="572" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="573" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="574" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="575" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="576" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="577" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="578" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="579" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="580" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="581" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="582" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="583" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="584" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="585" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="586" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="587" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="588" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="589" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="590" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="591" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="592" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="593" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="594" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="595" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="596" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="597" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="598" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="599" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="600" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="601" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="602" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="603" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="604" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="605" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="606" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="607" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="608" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="609" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="610" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="611" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="612" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="613" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="614" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="615" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="616" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="617" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="618" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="619" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="620" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="621" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="622" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="623" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="624" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="625" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="626" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="627" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="628" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="629" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="630" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="631" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="632" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="633" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="634" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="635" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="636" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="637" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="638" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="639" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="640" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="641" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="642" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="643" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="644" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="645" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="646" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="647" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="648" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="649" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="650" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="651" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="652" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="653" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="654" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="655" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="656" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="657" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="658" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="659" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="660" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="661" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="662" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="663" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="664" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="665" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="666" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="667" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="668" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="669" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="670" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="671" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="672" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="673" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="674" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="675" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="676" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="677" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="678" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="679" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="680" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="681" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="682" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="683" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="684" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="685" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="686" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="687" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="688" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="689" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="690" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="691" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="692" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="693" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="694" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="695" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="696" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="697" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="698" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="699" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="700" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="701" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="702" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="703" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="704" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="705" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="706" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="707" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="708" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="709" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="710" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="711" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="712" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="713" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="714" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="715" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="716" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="717" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="718" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="719" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="720" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="721" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="722" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="723" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="724" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="725" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="726" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="727" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="728" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="729" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="730" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="731" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="732" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="733" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="734" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="735" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="736" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="737" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="738" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="739" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="740" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="741" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="742" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="743" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="744" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="745" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="746" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="747" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="748" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="749" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="750" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="751" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="752" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="753" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="754" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="755" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="756" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="757" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="758" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="759" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="760" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="761" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="762" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="763" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="764" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="765" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="766" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="767" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="768" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="769" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="770" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="771" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="772" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="773" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="774" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="775" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="776" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="777" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="778" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="779" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="780" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="781" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="782" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="783" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="784" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="785" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="786" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="787" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="788" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="789" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="790" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="791" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="792" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="793" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="794" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="795" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="796" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="797" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="798" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="799" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="800" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="801" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="802" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="803" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="804" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="805" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="806" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="807" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="808" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="809" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="810" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="811" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="812" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="813" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="814" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="815" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="816" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="817" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="818" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="819" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="820" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="821" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="822" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="823" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="824" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="825" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="826" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="827" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="828" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="829" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="830" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="831" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="832" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="833" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="834" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="835" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="836" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="837" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="838" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="839" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="840" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="841" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="842" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="843" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="844" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="845" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="846" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="847" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="848" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="849" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="850" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="851" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="852" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="853" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="854" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="855" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="856" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="857" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="858" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="859" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="860" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="861" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="862" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="863" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="864" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="865" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="866" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="867" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="868" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="869" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="870" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="871" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="872" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="873" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="874" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="875" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="876" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="877" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="878" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="879" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="880" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="881" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="882" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="883" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="884" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="885" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="886" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="887" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="888" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="889" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="890" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="891" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="892" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="893" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="894" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="895" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="896" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="897" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="898" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="899" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="900" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="901" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="902" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="903" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="904" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="905" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="906" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="907" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="908" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="909" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="910" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="911" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="912" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="913" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="914" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="915" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="916" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="917" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="918" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="919" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="920" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="921" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="922" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="923" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="924" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="925" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="926" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="927" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="928" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="929" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="930" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="931" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="932" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="933" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="934" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="935" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="936" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="937" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="938" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="939" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="940" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="941" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="942" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="943" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="944" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="945" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="946" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="947" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="948" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="949" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="950" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="951" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="952" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="953" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="954" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="955" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="956" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="957" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="958" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="959" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="960" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="961" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="962" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="963" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="964" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="965" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="966" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="967" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="968" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="969" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="970" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="971" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="972" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="973" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="974" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="975" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="976" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="977" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="978" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="979" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="980" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="981" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="982" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="983" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="984" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="985" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="986" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="987" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="988" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="989" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="990" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="991" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="992" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="993" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="994" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="995" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="996" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="997" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="998" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <autoFilter ref="A1:I34" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>